<commit_message>
day 2 simple excel charts and data structuring
</commit_message>
<xml_diff>
--- a/excel/insurance.xlsx
+++ b/excel/insurance.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\JN1PEPF000031D8\EXCELCNV\30eb5b39-8db6-4898-99f8-fcacb4c5efb0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C76AA66-C9B3-40C7-877F-A141269FE0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="168" documentId="8_{D6C84D97-BFAE-4595-A2E3-1A6CD903E8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B542502-EFC2-4CD5-841F-B25DF13AD844}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{A2CBA70D-2931-4E50-9D28-97BBB7F6DBA5}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" activeTab="3" xr2:uid="{A2CBA70D-2931-4E50-9D28-97BBB7F6DBA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Insured" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId2"/>
+    <sheet name="Charts" sheetId="4" r:id="rId3"/>
+    <sheet name="Notes" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -59,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4023" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4053" uniqueCount="40">
   <si>
     <t>age</t>
   </si>
@@ -111,12 +113,81 @@
   <si>
     <t>northeast</t>
   </si>
+  <si>
+    <t>stat</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Smoker count = 1338 * 0.205 = 274</t>
+  </si>
+  <si>
+    <t>Average Charge</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Smoker</t>
+  </si>
+  <si>
+    <t>Non-Smoker</t>
+  </si>
+  <si>
+    <t>Normal-weight</t>
+  </si>
+  <si>
+    <t>Overweight</t>
+  </si>
+  <si>
+    <t>Obese</t>
+  </si>
+  <si>
+    <t>Data Average relations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smoker </t>
+  </si>
+  <si>
+    <t>Much higher than</t>
+  </si>
+  <si>
+    <t>non-Smoker</t>
+  </si>
+  <si>
+    <t>Slightly higher than</t>
+  </si>
+  <si>
+    <t>obese</t>
+  </si>
+  <si>
+    <t>higher than</t>
+  </si>
+  <si>
+    <t>non-obese</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,6 +318,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -593,8 +671,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -660,6 +741,926 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Charts!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average Charge</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$2:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Male</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Female</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Smoker</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Non-Smoker</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Normal-weight</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Overweight</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Obese</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$B$2:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>13956.751177721886</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12569.578843835339</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>32050.231831532848</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8434.2682978561988</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10409.337708977779</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10987.509891318654</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15552.335468868452</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A509-442E-9EF6-BFDC1E76BC62}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="26070024"/>
+        <c:axId val="26362888"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="26070024"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="26362888"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="26362888"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="26070024"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CD8666B-3D0D-E0EA-620F-A30EEAC72A78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C9A1064-6057-4613-9ADA-9B437352E3F2}" name="Insured" displayName="Insured" ref="A1:I1339" totalsRowShown="0">
   <autoFilter ref="A1:I1339" xr:uid="{0C9A1064-6057-4613-9ADA-9B437352E3F2}"/>
@@ -677,6 +1678,21 @@
     <tableColumn id="9" xr3:uid="{FF9A16F9-15D9-44C9-AF45-D22AE9895BFF}" name="bmi_class" dataDxfId="0">
       <calculatedColumnFormula array="1">_xlfn.IFS(Insured[[#This Row],[bmi]]&lt;18.5,"underweight",Insured[[#This Row],[bmi]]&lt;25,"normal",Insured[[#This Row],[bmi]]&lt;30,"overweight",TRUE,"obese")</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6065E84D-B1CC-4342-B27E-D240D46B9075}" name="Table2" displayName="Table2" ref="A1:F6" totalsRowShown="0">
+  <autoFilter ref="A1:F6" xr:uid="{6065E84D-B1CC-4342-B27E-D240D46B9075}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{1467D690-2BF1-4776-8913-298E579A4C21}" name="stat"/>
+    <tableColumn id="2" xr3:uid="{ADF72713-CA50-462F-842B-ECA539B09A3F}" name="age"/>
+    <tableColumn id="3" xr3:uid="{B46CA205-8784-4C60-A8F9-A2A97E109731}" name="bmi"/>
+    <tableColumn id="4" xr3:uid="{039B781F-F414-4CDD-9D4F-24368FBC5B16}" name="children"/>
+    <tableColumn id="5" xr3:uid="{4F590CFE-0648-4B9F-BD74-E1D2E721D0DC}" name="charges"/>
+    <tableColumn id="6" xr3:uid="{DBC549F9-22EA-4A92-BBD2-C39E37413B78}" name="smoker_flag"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -42508,10 +43524,311 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED511D6-6F4F-4E15-90F5-2D3EFBA423E0}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2">
+        <f>AVERAGE(Insured[age])</f>
+        <v>39.207025411061288</v>
+      </c>
+      <c r="C2">
+        <f>AVERAGE(Insured[bmi])</f>
+        <v>30.663396860986538</v>
+      </c>
+      <c r="D2">
+        <f>AVERAGE(Insured[children])</f>
+        <v>1.0949177877428999</v>
+      </c>
+      <c r="E2">
+        <f>AVERAGE(Insured[charges])</f>
+        <v>13270.422265141257</v>
+      </c>
+      <c r="F2">
+        <f>AVERAGE(Insured[smoker_flag])</f>
+        <v>0.20478325859491778</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <f>MEDIAN(Insured[age])</f>
+        <v>39</v>
+      </c>
+      <c r="C3">
+        <f>MEDIAN(Insured[bmi])</f>
+        <v>30.4</v>
+      </c>
+      <c r="D3">
+        <f>MEDIAN(Insured[children])</f>
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <f>MEDIAN(Insured[charges])</f>
+        <v>9382.0329999999994</v>
+      </c>
+      <c r="F3">
+        <f>MEDIAN(Insured[smoker_flag])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <f>MIN(Insured[age])</f>
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <f>MIN(Insured[bmi])</f>
+        <v>15.96</v>
+      </c>
+      <c r="D4">
+        <f>MIN(Insured[children])</f>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <f>MIN(Insured[charges])</f>
+        <v>1121.8739</v>
+      </c>
+      <c r="F4">
+        <f>MIN(Insured[smoker_flag])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <f>MAX(Insured[age])</f>
+        <v>64</v>
+      </c>
+      <c r="C5">
+        <f>MAX(Insured[bmi])</f>
+        <v>53.13</v>
+      </c>
+      <c r="D5">
+        <f>MAX(Insured[children])</f>
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <f>MAX(Insured[charges])</f>
+        <v>63770.428010000003</v>
+      </c>
+      <c r="F5">
+        <f>MAX(Insured[smoker_flag])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6">
+        <f>COUNT(Insured[age])</f>
+        <v>1338</v>
+      </c>
+      <c r="C6">
+        <f>COUNT(Insured[bmi])</f>
+        <v>1338</v>
+      </c>
+      <c r="D6">
+        <f>COUNT(Insured[children])</f>
+        <v>1338</v>
+      </c>
+      <c r="E6">
+        <f>COUNT(Insured[charges])</f>
+        <v>1338</v>
+      </c>
+      <c r="F6">
+        <f>COUNT(Insured[smoker_flag])</f>
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E02E57D-B597-409A-AA63-D59395B6D4FA}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2">
+        <f>AVERAGEIF(Insured[sex],"male",Insured[charges])</f>
+        <v>13956.751177721886</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3">
+        <f>AVERAGEIF(Insured[sex],"female",Insured[charges])</f>
+        <v>12569.578843835339</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <f>AVERAGEIF(Insured[smoker],"yes",Insured[charges])</f>
+        <v>32050.231831532848</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5">
+        <f>AVERAGEIF(Insured[smoker],"no",Insured[charges])</f>
+        <v>8434.2682978561988</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <f>AVERAGEIF(Insured[bmi_class],"normal",Insured[charges])</f>
+        <v>10409.337708977779</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7">
+        <f>AVERAGEIF(Insured[bmi_class],"overweight",Insured[charges])</f>
+        <v>10987.509891318654</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8">
+        <f>AVERAGEIF(Insured[bmi_class],"obese",Insured[charges])</f>
+        <v>15552.335468868452</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2060717-9766-4C1C-8A8A-7E4FD3282861}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>